<commit_message>
Agregada funcionalidad para subir casos de prueba a JIRA/QMetry
</commit_message>
<xml_diff>
--- a/casos de prueba/plantilla_base.xlsx
+++ b/casos de prueba/plantilla_base.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://everisgroup-my.sharepoint.com/personal/dnarvaec_emeal_nttdata_com1/Documents/Documents/Proyectos AUTO/Importar a JIRA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://everisgroup-my.sharepoint.com/personal/dnarvaec_emeal_nttdata_com1/Documents/Documents/Proyectos AUTO/Everest/auto-api-axet-plugin/demo-servicios-axet-plugin/casos de prueba/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="424" documentId="13_ncr:1_{8745CEFB-2D26-495B-BC07-20C89885C5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A806503F-9501-4FFC-A0C1-DB1FBF934876}"/>
+  <xr:revisionPtr revIDLastSave="441" documentId="13_ncr:1_{8745CEFB-2D26-495B-BC07-20C89885C5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96455551-13AD-465C-A2CE-35DB5223CE2B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="41">
   <si>
     <t>Resultado Esperado</t>
   </si>
@@ -141,58 +141,13 @@
     <t>Resultado Final 7</t>
   </si>
   <si>
-    <t>Accion 1</t>
-  </si>
-  <si>
-    <t>Datos 1</t>
-  </si>
-  <si>
-    <t>Resultado Esperado 1</t>
-  </si>
-  <si>
-    <t>Accion 2</t>
-  </si>
-  <si>
-    <t>Accion 3</t>
-  </si>
-  <si>
-    <t>Accion 4</t>
-  </si>
-  <si>
-    <t>Accion 5</t>
-  </si>
-  <si>
-    <t>Accion 6</t>
-  </si>
-  <si>
-    <t>Datos 2</t>
-  </si>
-  <si>
-    <t>Datos 3</t>
-  </si>
-  <si>
-    <t>Datos 4</t>
-  </si>
-  <si>
-    <t>Datos 5</t>
-  </si>
-  <si>
-    <t>Datos 6</t>
-  </si>
-  <si>
-    <t>Resultado Esperado 2</t>
-  </si>
-  <si>
-    <t>Resultado Esperado 3</t>
-  </si>
-  <si>
-    <t>Resultado Esperado 4</t>
-  </si>
-  <si>
-    <t>Resultado Esperado 5</t>
-  </si>
-  <si>
-    <t>Resultado Esperado 6</t>
+    <t xml:space="preserve">Datos </t>
+  </si>
+  <si>
+    <t>Acciones</t>
+  </si>
+  <si>
+    <t>Resultados Esperados</t>
   </si>
 </sst>
 </file>
@@ -548,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D519161F-1F8E-4CF9-9D0E-F42322125AF5}">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.08984375" customWidth="1"/>
@@ -607,10 +562,10 @@
         <v>31</v>
       </c>
       <c r="G2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H2" t="s">
         <v>38</v>
-      </c>
-      <c r="H2" t="s">
-        <v>39</v>
       </c>
       <c r="I2" t="s">
         <v>40</v>
@@ -618,428 +573,176 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H3" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="I3" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>33</v>
       </c>
       <c r="G4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H4" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="I4" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H5" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="I5" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" t="s">
+        <v>35</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H6" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="I6" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="H7" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="I7" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G8" t="s">
+        <v>39</v>
+      </c>
+      <c r="H8" t="s">
         <v>38</v>
-      </c>
-      <c r="H8" t="s">
-        <v>39</v>
       </c>
       <c r="I8" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>2</v>
-      </c>
-      <c r="G9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H9" t="s">
-        <v>46</v>
-      </c>
-      <c r="I9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="G10" t="s">
-        <v>42</v>
-      </c>
-      <c r="H10" t="s">
-        <v>47</v>
-      </c>
-      <c r="I10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>2</v>
-      </c>
-      <c r="G11" t="s">
-        <v>43</v>
-      </c>
-      <c r="H11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <v>2</v>
-      </c>
-      <c r="G12" t="s">
-        <v>44</v>
-      </c>
-      <c r="H12" t="s">
-        <v>49</v>
-      </c>
-      <c r="I12" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" t="s">
-        <v>26</v>
-      </c>
-      <c r="F13" t="s">
-        <v>33</v>
-      </c>
-      <c r="G13" t="s">
-        <v>38</v>
-      </c>
-      <c r="H13" t="s">
-        <v>39</v>
-      </c>
-      <c r="I13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <v>3</v>
-      </c>
-      <c r="G14" t="s">
-        <v>41</v>
-      </c>
-      <c r="H14" t="s">
-        <v>46</v>
-      </c>
-      <c r="I14" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <v>3</v>
-      </c>
-      <c r="G15" t="s">
-        <v>42</v>
-      </c>
-      <c r="H15" t="s">
-        <v>47</v>
-      </c>
-      <c r="I15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16">
-        <v>4</v>
-      </c>
-      <c r="B16" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" t="s">
-        <v>34</v>
-      </c>
-      <c r="G16" t="s">
-        <v>38</v>
-      </c>
-      <c r="H16" t="s">
-        <v>39</v>
-      </c>
-      <c r="I16" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17">
-        <v>4</v>
-      </c>
-      <c r="G17" t="s">
-        <v>41</v>
-      </c>
-      <c r="H17" t="s">
-        <v>46</v>
-      </c>
-      <c r="I17" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18">
-        <v>4</v>
-      </c>
-      <c r="G18" t="s">
-        <v>42</v>
-      </c>
-      <c r="H18" t="s">
-        <v>47</v>
-      </c>
-      <c r="I18" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A19">
-        <v>5</v>
-      </c>
-      <c r="B19" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E19" t="s">
-        <v>28</v>
-      </c>
-      <c r="F19" t="s">
-        <v>35</v>
-      </c>
-      <c r="G19" t="s">
-        <v>38</v>
-      </c>
-      <c r="H19" t="s">
-        <v>39</v>
-      </c>
-      <c r="I19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20">
-        <v>5</v>
-      </c>
-      <c r="G20" t="s">
-        <v>41</v>
-      </c>
-      <c r="H20" t="s">
-        <v>46</v>
-      </c>
-      <c r="I20" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <v>6</v>
-      </c>
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" t="s">
-        <v>29</v>
-      </c>
-      <c r="F21" t="s">
-        <v>36</v>
-      </c>
-      <c r="G21" t="s">
-        <v>38</v>
-      </c>
-      <c r="H21" t="s">
-        <v>39</v>
-      </c>
-      <c r="I21" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <v>6</v>
-      </c>
-      <c r="G22" t="s">
-        <v>41</v>
-      </c>
-      <c r="H22" t="s">
-        <v>46</v>
-      </c>
-      <c r="I22" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <v>6</v>
-      </c>
-      <c r="G23" t="s">
-        <v>42</v>
-      </c>
-      <c r="H23" t="s">
-        <v>47</v>
-      </c>
-      <c r="I23" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A24">
-        <v>7</v>
-      </c>
-      <c r="B24" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" t="s">
-        <v>16</v>
-      </c>
-      <c r="D24" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" t="s">
-        <v>30</v>
-      </c>
-      <c r="F24" t="s">
-        <v>37</v>
-      </c>
-      <c r="G24" t="s">
-        <v>38</v>
-      </c>
-      <c r="H24" t="s">
-        <v>39</v>
-      </c>
-      <c r="I24" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A25">
-        <v>7</v>
-      </c>
-      <c r="G25" t="s">
-        <v>41</v>
-      </c>
-      <c r="H25" t="s">
-        <v>46</v>
-      </c>
-      <c r="I25" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>7</v>
-      </c>
-      <c r="G26" t="s">
-        <v>42</v>
-      </c>
-      <c r="H26" t="s">
-        <v>47</v>
-      </c>
-      <c r="I26" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>